<commit_message>
Update - March 2026
</commit_message>
<xml_diff>
--- a/ECB_mean.xlsx
+++ b/ECB_mean.xlsx
@@ -69,7 +69,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:C65"/>
+  <dimension ref="A1:C74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -131,7 +131,7 @@
         <v>43983</v>
       </c>
       <c r="B7" s="2">
-        <v>3.681066406503593</v>
+        <v>3.6810664065035921</v>
       </c>
       <c r="C7" s="2">
         <v>2</v>
@@ -197,7 +197,7 @@
         <v>44166</v>
       </c>
       <c r="B13" s="2">
-        <v>3.572021069962886</v>
+        <v>3.5720210699628878</v>
       </c>
       <c r="C13" s="2">
         <v>2</v>
@@ -285,7 +285,7 @@
         <v>44409</v>
       </c>
       <c r="B21" s="2">
-        <v>3.8924362002853607</v>
+        <v>3.8924362002853692</v>
       </c>
       <c r="C21" s="2">
         <v>2.5</v>
@@ -340,7 +340,7 @@
         <v>44562</v>
       </c>
       <c r="B26" s="2">
-        <v>4.906882975223958</v>
+        <v>4.9068829752239349</v>
       </c>
       <c r="C26" s="2">
         <v>4.5999999046325684</v>
@@ -373,7 +373,7 @@
         <v>44652</v>
       </c>
       <c r="B29" s="2">
-        <v>7.5673831320844851</v>
+        <v>7.5673831320844904</v>
       </c>
       <c r="C29" s="2">
         <v>6.6999998092651367</v>
@@ -395,7 +395,7 @@
         <v>44713</v>
       </c>
       <c r="B31" s="2">
-        <v>7.0988523981729088</v>
+        <v>7.098852398172915</v>
       </c>
       <c r="C31" s="2">
         <v>6</v>
@@ -406,7 +406,7 @@
         <v>44743</v>
       </c>
       <c r="B32" s="2">
-        <v>6.8909852014929909</v>
+        <v>6.8909852014929864</v>
       </c>
       <c r="C32" s="2">
         <v>5.9000000953674316</v>
@@ -439,7 +439,7 @@
         <v>44835</v>
       </c>
       <c r="B35" s="2">
-        <v>7.113767751951821</v>
+        <v>7.1137677519518201</v>
       </c>
       <c r="C35" s="2">
         <v>6</v>
@@ -571,7 +571,7 @@
         <v>45200</v>
       </c>
       <c r="B47" s="2">
-        <v>5.0584100961271883</v>
+        <v>5.0584100961271838</v>
       </c>
       <c r="C47" s="2">
         <v>5</v>
@@ -626,7 +626,7 @@
         <v>45352</v>
       </c>
       <c r="B52" s="2">
-        <v>4.3897269615596946</v>
+        <v>4.3897269615596954</v>
       </c>
       <c r="C52" s="2">
         <v>3.5</v>
@@ -648,7 +648,7 @@
         <v>45413</v>
       </c>
       <c r="B54" s="2">
-        <v>4.2578411739050264</v>
+        <v>4.2578411739050255</v>
       </c>
       <c r="C54" s="2">
         <v>3</v>
@@ -768,8 +768,107 @@
       <c r="A65" s="1">
         <v>45748</v>
       </c>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
+      <c r="B65" s="2">
+        <v>5.1107342056204654</v>
+      </c>
+      <c r="C65" s="2">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="1">
+        <v>45778</v>
+      </c>
+      <c r="B66" s="2">
+        <v>4.9675351187251602</v>
+      </c>
+      <c r="C66" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="1">
+        <v>45809</v>
+      </c>
+      <c r="B67" s="2">
+        <v>4.4501922887229615</v>
+      </c>
+      <c r="C67" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="1">
+        <v>45839</v>
+      </c>
+      <c r="B68" s="2">
+        <v>4.3660442167723472</v>
+      </c>
+      <c r="C68" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="1">
+        <v>45870</v>
+      </c>
+      <c r="B69" s="2">
+        <v>4.3121425799448758</v>
+      </c>
+      <c r="C69" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="1">
+        <v>45901</v>
+      </c>
+      <c r="B70" s="2">
+        <v>4.4544923336211895</v>
+      </c>
+      <c r="C70" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="1">
+        <v>45931</v>
+      </c>
+      <c r="B71" s="2">
+        <v>4.4864942500958236</v>
+      </c>
+      <c r="C71" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" s="1">
+        <v>45962</v>
+      </c>
+      <c r="B72" s="2">
+        <v>4.6565247137459655</v>
+      </c>
+      <c r="C72" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" s="1">
+        <v>45992</v>
+      </c>
+      <c r="B73" s="2">
+        <v>4.3801899369403978</v>
+      </c>
+      <c r="C73" s="2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="1">
+        <v>46023</v>
+      </c>
+      <c r="B74" s="2"/>
+      <c r="C74" s="2"/>
     </row>
   </sheetData>
 </worksheet>

</xml_diff>